<commit_message>
EU and OFAC v6
</commit_message>
<xml_diff>
--- a/record-linkage-of-ofac-and-eu-sanctions-lists/text-embeddings/text_embeddings_confusion_matrix.xlsx
+++ b/record-linkage-of-ofac-and-eu-sanctions-lists/text-embeddings/text_embeddings_confusion_matrix.xlsx
@@ -376,7 +376,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11.03"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="6.58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="7.69"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8.8"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="17.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="23.97"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="9.08"/>
@@ -437,37 +437,37 @@
         <v>0.7</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>2102</v>
+        <v>2125</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>43871</v>
+        <v>342543</v>
       </c>
       <c r="E2" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>31834048</v>
+        <v>31535376</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>0.0457224892871903</v>
+        <v>0.00616535332551905</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>0.98731798966651</v>
+        <v>0.998121183654298</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>0.998623025912634</v>
+        <v>0.989255129101437</v>
       </c>
       <c r="L2" s="4" t="n">
-        <v>0.087397613404848</v>
-      </c>
-      <c r="M2" s="0" t="n">
-        <v>0.8</v>
+        <v>0.012255007972964</v>
+      </c>
+      <c r="M2" s="2" t="n">
+        <v>0.7</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -478,37 +478,37 @@
         <v>0.75</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>2102</v>
+        <v>2118</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>43871</v>
+        <v>141888</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>31834048</v>
+        <v>31736031</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>0.0457224892871903</v>
+        <v>0.0147077205116454</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>0.98731798966651</v>
+        <v>0.994833255049319</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>0.998623025912634</v>
+        <v>0.99554897156993</v>
       </c>
       <c r="L3" s="4" t="n">
-        <v>0.087397613404848</v>
-      </c>
-      <c r="M3" s="0" t="n">
-        <v>0.8</v>
+        <v>0.0289868956786533</v>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>0.7</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -525,10 +525,10 @@
         <v>43871</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>27</v>
@@ -548,8 +548,8 @@
       <c r="L4" s="4" t="n">
         <v>0.087397613404848</v>
       </c>
-      <c r="M4" s="0" t="n">
-        <v>0.8</v>
+      <c r="M4" s="2" t="n">
+        <v>0.7</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -566,10 +566,10 @@
         <v>9213</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>57</v>
@@ -589,8 +589,8 @@
       <c r="L5" s="4" t="n">
         <v>0.308930967645743</v>
       </c>
-      <c r="M5" s="0" t="n">
-        <v>0.8</v>
+      <c r="M5" s="2" t="n">
+        <v>0.7</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -607,10 +607,10 @@
         <v>1206</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>124</v>
@@ -630,8 +630,8 @@
       <c r="L6" s="4" t="n">
         <v>0.750936329588015</v>
       </c>
-      <c r="M6" s="0" t="n">
-        <v>0.8</v>
+      <c r="M6" s="2" t="n">
+        <v>0.7</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -648,10 +648,10 @@
         <v>161</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>263</v>
+        <v>286</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="G7" s="3" t="n">
         <v>290</v>
@@ -671,8 +671,8 @@
       <c r="L7" s="4" t="n">
         <v>0.890772584160814</v>
       </c>
-      <c r="M7" s="0" t="n">
-        <v>0.8</v>
+      <c r="M7" s="2" t="n">
+        <v>0.7</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -689,10 +689,10 @@
         <v>57</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>1046</v>
+        <v>1069</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>1073</v>
@@ -712,8 +712,8 @@
       <c r="L8" s="4" t="n">
         <v>0.651449722393584</v>
       </c>
-      <c r="M8" s="0" t="n">
-        <v>0.8</v>
+      <c r="M8" s="2" t="n">
+        <v>0.7</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -753,7 +753,7 @@
       <c r="L9" s="4" t="n">
         <v>0.110116999311769</v>
       </c>
-      <c r="M9" s="0" t="n">
+      <c r="M9" s="2" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -794,7 +794,7 @@
       <c r="L10" s="4" t="n">
         <v>0.200257039373759</v>
       </c>
-      <c r="M10" s="0" t="n">
+      <c r="M10" s="2" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -835,7 +835,7 @@
       <c r="L11" s="4" t="n">
         <v>0.352690916826207</v>
       </c>
-      <c r="M11" s="0" t="n">
+      <c r="M11" s="2" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -876,7 +876,7 @@
       <c r="L12" s="4" t="n">
         <v>0.540837336993823</v>
       </c>
-      <c r="M12" s="0" t="n">
+      <c r="M12" s="2" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -917,7 +917,7 @@
       <c r="L13" s="4" t="n">
         <v>0.706963249516441</v>
       </c>
-      <c r="M13" s="0" t="n">
+      <c r="M13" s="2" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -958,7 +958,7 @@
       <c r="L14" s="4" t="n">
         <v>0.756410256410256</v>
       </c>
-      <c r="M14" s="0" t="n">
+      <c r="M14" s="2" t="n">
         <v>0.7</v>
       </c>
     </row>
@@ -999,7 +999,7 @@
       <c r="L15" s="4" t="n">
         <v>0.553663952627683</v>
       </c>
-      <c r="M15" s="0" t="n">
+      <c r="M15" s="2" t="n">
         <v>0.7</v>
       </c>
     </row>

</xml_diff>